<commit_message>
Backlink plan: Profiles tab (social + company databases)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2g112JF6CCLo8Tg7CRZKC
</commit_message>
<xml_diff>
--- a/docs/seo/Swansura_Backlink_Plan_2026-10-28.xlsx
+++ b/docs/seo/Swansura_Backlink_Plan_2026-10-28.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlink plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pitch templates" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avoid" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pitch templates" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avoid" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlink plan'!$A$1:$O$32</definedName>
@@ -2713,6 +2714,726 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Link type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Done (URL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Companies House</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>https://find-and-update.company-information.service.gov.uk/company/16575553</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Registered (checked 28 Oct)</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Not a backlink, but the source every company database copies. UK law (Companies Act 2006 / Company, LLP and Business Names Regs 2015) also needs the registered name, number, place of registration (England &amp; Wales) and registered office on the website: add them to the footer legal line.</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Crunchbase</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>To create</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Free company profile: SWANSURA LTD (company no. 16575553), website, logo, founded July 2025, London, category Beauty / E-commerce, short description.</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>nofollow (brand signal)</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn company page</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/setup/new/</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>To create</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Company page with website, logo, industry Retail / Personal Care, location London; founder lists Swansura as employer.</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Dun &amp; Bradstreet D-U-N-S number</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>https://www.dnb.co.uk/duns-number.html</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>To request (free)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Free D-U-N-S number for the Ltd; adds a trusted business record and is needed for Apple Business Connect / Apple developer accounts.</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>no link (trust record)</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>F6S</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>https://www.f6s.com</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>To create</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Free startup profile with website; also lists programmes and deals.</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>profile link</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Endole / company-data mirrors</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>https://www.endole.co.uk</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Auto from Companies House</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Profiles appear automatically; where a free claim is offered, add the website and logo. Do not pay for upgrades.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>varies</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Tracxn / ZoomInfo / Owler</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.tracxn.com</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Auto / optional</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Company databases that pick up profiles from the web; check once and add the website if a free edit is allowed.</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Wellfound (AngelList)</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>https://wellfound.com</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Only if hiring or raising</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Skip unless hiring or fundraising.</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Startup media</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>YourStory (India)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>https://yourstory.com</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Pitch</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Story angle for Indian startup media: Indian natural brands Deyga and Vilvah reach UK customers through a London partner (Swansura). Use their story-submission route; give facts only (no sales figures you don't want public).</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>editorial, often dofollow</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Startup media</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Inc42 (India)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>https://inc42.com</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Pitch</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Same angle (Indian D2C brands going global via UK partners); offer a founder quote.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>editorial</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Startup media</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Startups.co.uk</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.startups.co.uk</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Pitch</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>UK small-business media; founder story of a new London beauty e-commerce company (2025).</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>editorial</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Startup media</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>UK Business Forums</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ukbusinessforums.co.uk</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Free member profile with website; take part genuinely, no link drops.</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Instagram @swansura_thebodystudio</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/swansura_thebodystudio</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Exists (linked in footer)</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Website in bio; Instagram Shopping via the Facebook &amp; Instagram channel.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/share/16wUrverHK/</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Website field, Shop tab, category Health/beauty.</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>TikTok @swansurathebodysh</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@swansurathebodysh</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Exists – rename</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Business account + website link. Rename the handle: "the body shop" is The Body Shop's trademark and not the brand ("The Body Studio").</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>YouTube @SwansuraThebodyshop</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@SwansuraThebodyshop</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Exists – rename</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Add the website to channel links. Rename the handle for the same trademark reason.</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Pinterest business</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>https://business.pinterest.com</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>To create</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Claim swansura.com, connect the Shopify catalogue (Pinterest sales channel) for product pins: real traffic for beauty and gifts.</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>nofollow + traffic</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>https://x.com</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>To create</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Needed to answer #journorequest; website in bio.</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.threads.net</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>To create</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>One tap from Instagram.</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>nofollow</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>sameAs + footer icons</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>https://www.swansura.com</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>To do (theme)</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>List every profile in the Organization schema sameAs and show the icons in the footer (live footer and schema list only Instagram).</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2787,7 +3508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>